<commit_message>
update: 77 cases - add backpack/equipment/settings/death/levelup systems
</commit_message>
<xml_diff>
--- a/test-cases/Flare主界面与功能测试用例.xlsx
+++ b/test-cases/Flare主界面与功能测试用例.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$I$78</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="24">
     <font>
       <name val="等线"/>
       <charset val="134"/>
@@ -37,25 +37,6 @@
       <name val="微软雅黑"/>
       <charset val="134"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <color rgb="FFFF0000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="等线"/>
-      <charset val="134"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="等线"/>
@@ -203,10 +184,16 @@
     </font>
     <font>
       <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="41">
     <fill>
       <patternFill/>
     </fill>
@@ -425,6 +412,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FF6B6B"/>
         <bgColor rgb="00FF6B6B"/>
       </patternFill>
@@ -589,137 +582,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="7" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="36" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -733,55 +726,32 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="37" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="39" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="39" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="40" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1169,7 +1139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -1177,100 +1147,101 @@
     <col width="32" customWidth="1" style="1" min="3" max="3"/>
     <col width="8" customWidth="1" style="1" min="4" max="4"/>
     <col width="12" customWidth="1" style="1" min="5" max="6"/>
-    <col width="28" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="6" max="6"/>
+    <col width="30" customWidth="1" style="1" min="7" max="7"/>
     <col width="38" customWidth="1" style="1" min="8" max="8"/>
     <col width="48" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>测试序列</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>测试模块</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>测试点</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>测试类型</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>版本号</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="10" t="inlineStr">
         <is>
           <t>前置条件</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="10" t="inlineStr">
         <is>
           <t>操作步骤</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="10" t="inlineStr">
         <is>
           <t>预期结果</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="65" customHeight="1" s="1">
-      <c r="A2" s="20" t="inlineStr">
+    <row r="2" ht="72" customHeight="1" s="1">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Main_UI_001</t>
         </is>
       </c>
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>主界面</t>
         </is>
       </c>
-      <c r="C2" s="20" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>冷启动-主界面完整展示</t>
         </is>
       </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E2" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F2" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>游戏已安装</t>
         </is>
       </c>
-      <c r="H2" s="20" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>点击桌面图标启动游戏</t>
         </is>
       </c>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>1. 游戏正常启动，主界面在合理时间内加载完成
 2. 界面包含【开始游戏】【设置】【退出】【致谢】按钮
@@ -1278,611 +1249,611 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="65" customHeight="1" s="1">
-      <c r="A3" s="20" t="inlineStr">
+    <row r="3" ht="72" customHeight="1" s="1">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Main_UI_002</t>
         </is>
       </c>
-      <c r="B3" s="20" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>主界面</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>各功能按钮点击响应</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>游戏启动成功，停留在主界面</t>
         </is>
       </c>
-      <c r="H3" s="20" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>依次点击【开始游戏】【设置】【退出】【致谢】</t>
         </is>
       </c>
-      <c r="I3" s="20" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>每个按钮点击后正确跳转到对应界面，无闪退、无卡死</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="65" customHeight="1" s="1">
-      <c r="A4" s="20" t="inlineStr">
+    <row r="4" ht="72" customHeight="1" s="1">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Main_UI_003</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>主界面</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>窗口缩放与分辨率适配</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>兼容性测试</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>游戏已启动</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>1. 拉伸窗口至不同尺寸
 2. 切换不同分辨率
 3. 观察UI布局</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>所有UI元素无重叠、无裁切、无拉伸变形，按钮仍可正常点击</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="65" customHeight="1" s="1">
-      <c r="A5" s="20" t="inlineStr">
+    <row r="5" ht="72" customHeight="1" s="1">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Main_UI_004</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>游戏已启动</t>
         </is>
       </c>
-      <c r="H5" s="20" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>1. 点击【开始游戏】
 2. 在角色选择界面点击【创建角色】</t>
         </is>
       </c>
-      <c r="I5" s="20" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面，显示：职业选择项、名称输入框、头像选择、【创建】与【取消】按钮</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="65" customHeight="1" s="1">
-      <c r="A6" s="20" t="inlineStr">
+    <row r="6" ht="72" customHeight="1" s="1">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Main_UI_005</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>职业选择-力士</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>选择职业【力士】</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>力士被高亮选中，显示力士的职业简介与主要属性说明</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="65" customHeight="1" s="1">
-      <c r="A7" s="20" t="inlineStr">
+    <row r="7" ht="72" customHeight="1" s="1">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Main_UI_006</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>职业选择-斥候</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>选择职业【斥候】</t>
         </is>
       </c>
-      <c r="I7" s="20" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>斥候被高亮选中，显示斥候的职业简介与主要属性说明</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="65" customHeight="1" s="1">
-      <c r="A8" s="20" t="inlineStr">
+    <row r="8" ht="72" customHeight="1" s="1">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Main_UI_007</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>职业选择-法师</t>
         </is>
       </c>
-      <c r="D8" s="22" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H8" s="20" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>选择职业【法师】</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>法师被高亮选中，显示法师的职业简介与主要属性说明</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="65" customHeight="1" s="1">
-      <c r="A9" s="20" t="inlineStr">
+    <row r="9" ht="72" customHeight="1" s="1">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Main_UI_008</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>名称输入-正常中英文</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H9" s="20" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>输入正常中英文名称（如艾琳、TestHero）</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>输入内容正确显示在输入框中，无乱码或截断</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="65" customHeight="1" s="1">
-      <c r="A10" s="20" t="inlineStr">
+    <row r="10" ht="72" customHeight="1" s="1">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Main_UI_009</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>名称输入-空名称</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>边界测试</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>不输入任何字符，点击【创建】</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>系统应有提示（名称不能为空）或自动使用默认名称，不应直接崩溃或创建无名角色</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="65" customHeight="1" s="1">
-      <c r="A11" s="20" t="inlineStr">
+    <row r="11" ht="72" customHeight="1" s="1">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Main_UI_010</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>名称输入-超长名称</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>边界测试</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H11" s="20" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>输入超过最大长度限制的名称</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr">
+      <c r="I11" s="11" t="inlineStr">
         <is>
           <t>名称被截断到最大长度，或系统给出长度提示，不应崩溃</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="65" customHeight="1" s="1">
-      <c r="A12" s="20" t="inlineStr">
+    <row r="12" ht="72" customHeight="1" s="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Main_UI_011</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>名称输入-特殊字符</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>边界测试</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H12" s="20" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>输入含特殊字符的名称（如 @#$%^&amp;*&lt;&gt;）</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>系统正常处理，不崩溃；若限制特殊字符应有明确提示</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="65" customHeight="1" s="1">
-      <c r="A13" s="20" t="inlineStr">
+    <row r="13" ht="72" customHeight="1" s="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Main_UI_012</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>默认名称（随机生成）</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H13" s="20" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>不输入名称，直接点击【创建】</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr">
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>系统自动生成默认名称，名称有效且可正常进入游戏</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="65" customHeight="1" s="1">
-      <c r="A14" s="20" t="inlineStr">
+    <row r="14" ht="72" customHeight="1" s="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Main_UI_013</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>创建-取消操作</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>异常测试</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>1. 输入名称并选择职业
 2. 点击【取消】</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>返回角色选择界面，未创建新角色，设置未保存</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="65" customHeight="1" s="1">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="15" ht="72" customHeight="1" s="1">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>Main_UI_014</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>死亡不可复活-勾选</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H15" s="20" t="inlineStr">
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t>1. 勾选「死亡不可复活」
 2. 创建角色进入游戏
@@ -1890,56 +1861,56 @@
 4. 观察死亡界面</t>
         </is>
       </c>
-      <c r="I15" s="20" t="inlineStr">
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>角色死亡后仅有【退出】选项有效，继续游戏选项不可点击或不存在</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="65" customHeight="1" s="1">
-      <c r="A16" s="20" t="inlineStr">
+    <row r="16" ht="72" customHeight="1" s="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Main_UI_015</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>创建-力士并进入游戏</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F16" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>1. 选择职业【力士】
 2. 使用默认名称
 3. 点击【创建】</t>
         </is>
       </c>
-      <c r="I16" s="20" t="inlineStr">
+      <c r="I16" s="11" t="inlineStr">
         <is>
           <t>1. 角色创建成功，进入游戏主界面
 2. 角色头顶名称与默认名称一致
@@ -1947,50 +1918,50 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="65" customHeight="1" s="1">
-      <c r="A17" s="20" t="inlineStr">
+    <row r="17" ht="72" customHeight="1" s="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Main_UI_016</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>创建-斥候并进入游戏</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H17" s="20" t="inlineStr">
+      <c r="H17" s="11" t="inlineStr">
         <is>
           <t>1. 选择职业【斥候】
 2. 使用默认名称
 3. 点击【创建】</t>
         </is>
       </c>
-      <c r="I17" s="20" t="inlineStr">
+      <c r="I17" s="11" t="inlineStr">
         <is>
           <t>1. 角色创建成功，进入游戏主界面
 2. 角色头顶名称与默认名称一致
@@ -1998,50 +1969,50 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="65" customHeight="1" s="1">
-      <c r="A18" s="20" t="inlineStr">
+    <row r="18" ht="72" customHeight="1" s="1">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Main_UI_017</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>角色创建</t>
         </is>
       </c>
-      <c r="C18" s="20" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>创建-法师并进入游戏</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
         <is>
           <t>进入角色创建界面</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>1. 选择职业【法师】
 2. 使用默认名称
 3. 点击【创建】</t>
         </is>
       </c>
-      <c r="I18" s="20" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>1. 角色创建成功，进入游戏主界面
 2. 角色头顶名称与默认名称一致
@@ -2049,531 +2020,531 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="65" customHeight="1" s="1">
-      <c r="A19" s="20" t="inlineStr">
+    <row r="19" ht="72" customHeight="1" s="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Main_UI_018</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>ESC菜单</t>
         </is>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>保存并退出</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F19" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>已创建角色并进入游戏</t>
         </is>
       </c>
-      <c r="H19" s="20" t="inlineStr">
+      <c r="H19" s="11" t="inlineStr">
         <is>
           <t>1. 按ESC
 2. 点击【保存并退出】</t>
         </is>
       </c>
-      <c r="I19" s="20" t="inlineStr">
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>1. 游戏退出到主界面
 2. 重新点击【开始游戏】，存档列表中显示该存档，确认数据已保存</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="65" customHeight="1" s="1">
-      <c r="A20" s="20" t="inlineStr">
+    <row r="20" ht="72" customHeight="1" s="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Main_UI_019</t>
         </is>
       </c>
-      <c r="B20" s="20" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>ESC菜单</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>取消返回游戏</t>
         </is>
       </c>
-      <c r="D20" s="22" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E20" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F20" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>游戏中按下ESC弹出菜单</t>
         </is>
       </c>
-      <c r="H20" s="20" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>1. 按ESC
 2. 点击【取消】或再次按ESC</t>
         </is>
       </c>
-      <c r="I20" s="20" t="inlineStr">
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>菜单关闭，正常返回游戏，游戏状态未受影响</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="65" customHeight="1" s="1">
-      <c r="A21" s="20" t="inlineStr">
+    <row r="21" ht="72" customHeight="1" s="1">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>Main_UI_020</t>
         </is>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>存档列表展示</t>
         </is>
       </c>
-      <c r="D21" s="22" t="inlineStr">
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E21" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F21" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G21" s="20" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
         <is>
           <t>已有至少一个存档</t>
         </is>
       </c>
-      <c r="H21" s="20" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>1. 在主界面点击【开始游戏】
 2. 观察存档列表</t>
         </is>
       </c>
-      <c r="I21" s="20" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>正确显示存档信息：游玩时间、职业、等级、名称、当前所在位置</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="65" customHeight="1" s="1">
-      <c r="A22" s="20" t="inlineStr">
+    <row r="22" ht="72" customHeight="1" s="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Main_UI_021</t>
         </is>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C22" s="20" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>载入存档-数据完整性</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F22" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G22" s="20" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>已有存档</t>
         </is>
       </c>
-      <c r="H22" s="20" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>1. 点击存档
 2. 点击【载入】
 3. 进入游戏后检查角色状态</t>
         </is>
       </c>
-      <c r="I22" s="20" t="inlineStr">
+      <c r="I22" s="11" t="inlineStr">
         <is>
           <t>角色等级、装备、背包物品、当前位置、任务进度与存档前完全一致</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="65" customHeight="1" s="1">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="23" ht="72" customHeight="1" s="1">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Main_UI_022</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>删除存档</t>
         </is>
       </c>
-      <c r="D23" s="22" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E23" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F23" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G23" s="20" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>已有存档</t>
         </is>
       </c>
-      <c r="H23" s="20" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>1. 选中一个存档
 2. 点击【删除】
 3. 确认删除</t>
         </is>
       </c>
-      <c r="I23" s="20" t="inlineStr">
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>存档从列表中移除，无法再载入</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="65" customHeight="1" s="1">
-      <c r="A24" s="20" t="inlineStr">
+    <row r="24" ht="72" customHeight="1" s="1">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Main_UI_023</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>删除存档-取消操作</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>异常测试</t>
         </is>
       </c>
-      <c r="F24" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G24" s="20" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
         <is>
           <t>已有存档，点击删除</t>
         </is>
       </c>
-      <c r="H24" s="20" t="inlineStr">
+      <c r="H24" s="11" t="inlineStr">
         <is>
           <t>1. 选中存档点击【删除】
 2. 在确认弹窗中选择【取消】</t>
         </is>
       </c>
-      <c r="I24" s="20" t="inlineStr">
+      <c r="I24" s="11" t="inlineStr">
         <is>
           <t>存档未被删除，仍在列表中</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="65" customHeight="1" s="1">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="25" ht="72" customHeight="1" s="1">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Main_UI_024</t>
         </is>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>多存档无冲突</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="D25" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E25" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G25" s="20" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>已创建多个不同职业的存档</t>
         </is>
       </c>
-      <c r="H25" s="20" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>1. 依次查看每个存档
 2. 逐一载入验证</t>
         </is>
       </c>
-      <c r="I25" s="20" t="inlineStr">
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>每个存档独立，角色信息正确，存档间无数据串扰</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="65" customHeight="1" s="1">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="26" ht="72" customHeight="1" s="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Main_UI_025</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>存档系统</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>新游戏-已有存档时创建新角色</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D26" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F26" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G26" s="20" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
         <is>
           <t>已有存档</t>
         </is>
       </c>
-      <c r="H26" s="20" t="inlineStr">
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t>1. 点击【新游戏】
 2. 完成角色创建</t>
         </is>
       </c>
-      <c r="I26" s="20" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>进入角色创建系统，新角色创建后与旧存档共存，互不影响</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="65" customHeight="1" s="1">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="27" ht="72" customHeight="1" s="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Main_UI_026</t>
         </is>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>游戏加载动画</t>
         </is>
       </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>游戏加载动画UI</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E27" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F27" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G27" s="20" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
         <is>
           <t>成功创建角色并进入游戏内</t>
         </is>
       </c>
-      <c r="H27" s="20" t="inlineStr">
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t>观察游戏加载动画是否正常</t>
         </is>
       </c>
-      <c r="I27" s="20" t="inlineStr">
+      <c r="I27" s="11" t="inlineStr">
         <is>
           <t>1.未出现动画UI丢失</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="67" customHeight="1" s="1">
-      <c r="A28" s="20" t="inlineStr">
+    <row r="28" ht="72" customHeight="1" s="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>Main_UI_027</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>游戏加载动画</t>
         </is>
       </c>
-      <c r="C28" s="20" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>游戏加载动画UI</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E28" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F28" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G28" s="20" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">成功创建角色并进入游戏内
 </t>
         </is>
       </c>
-      <c r="H28" s="20" t="inlineStr">
+      <c r="H28" s="11" t="inlineStr">
         <is>
           <t>1.切换不同分辨率与窗口化
 2.观察游戏加载动画是否正常</t>
         </is>
       </c>
-      <c r="I28" s="20" t="inlineStr">
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>2.未出现动画UI丢失</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1" s="1">
-      <c r="A29" s="20" t="inlineStr">
+    <row r="29" ht="72" customHeight="1" s="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Main_UI_028</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>游戏内界面UI</t>
         </is>
       </c>
-      <c r="C29" s="20" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>游戏内HUD展示-鼠标移动模式下</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E29" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F29" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G29" s="20" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
         <is>
           <t>成功创建角色并进入游戏内</t>
         </is>
       </c>
-      <c r="H29" s="20" t="inlineStr">
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t>观察游戏内界面UI界面是否完整</t>
         </is>
       </c>
-      <c r="I29" s="20" t="inlineStr">
+      <c r="I29" s="11" t="inlineStr">
         <is>
           <t>1.角色模型正常
 2.新手基本介绍正常出现
@@ -2581,49 +2552,49 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="56" customHeight="1" s="1">
-      <c r="A30" s="20" t="inlineStr">
+    <row r="30" ht="72" customHeight="1" s="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Main_UI_029</t>
         </is>
       </c>
-      <c r="B30" s="20" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>游戏内界面UI</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>游戏内HUD展示-多分辨率适配</t>
         </is>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E30" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F30" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G30" s="20" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
         <is>
           <t>成功创建角色并进入游戏内</t>
         </is>
       </c>
-      <c r="H30" s="20" t="inlineStr">
+      <c r="H30" s="11" t="inlineStr">
         <is>
           <t>1.切换不同分辨率与窗口化
 2.观察游戏内界面UI界面是否完整</t>
         </is>
       </c>
-      <c r="I30" s="20" t="inlineStr">
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>1.角色模型正常
 2.新手基本介绍正常出现
@@ -2631,385 +2602,385 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="28" customHeight="1" s="1">
-      <c r="A31" s="20" t="inlineStr">
+    <row r="31" ht="72" customHeight="1" s="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Main_UI_030</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>移动-鼠标点击可到达地形</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F31" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G31" s="20" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H31" s="20" t="inlineStr">
+      <c r="H31" s="11" t="inlineStr">
         <is>
           <t>1.点击左鼠标去可以去的地形
 2.观察角色是否移动到该地点</t>
         </is>
       </c>
-      <c r="I31" s="20" t="inlineStr">
+      <c r="I31" s="11" t="inlineStr">
         <is>
           <t>角色移动到该地点</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1" s="1">
-      <c r="A32" s="20" t="inlineStr">
+    <row r="32" ht="72" customHeight="1" s="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Main_UI_031</t>
         </is>
       </c>
-      <c r="B32" s="20" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>移动-鼠标点击不可到达地形（边界）</t>
         </is>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E32" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F32" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G32" s="20" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H32" s="20" t="inlineStr">
+      <c r="H32" s="11" t="inlineStr">
         <is>
           <t>1.点击左鼠标去不可以去的地形（地图边界）
 2.观察角色是否移动到该地点</t>
         </is>
       </c>
-      <c r="I32" s="20" t="inlineStr">
+      <c r="I32" s="11" t="inlineStr">
         <is>
           <t>角色原地未动</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="42" customHeight="1" s="1">
-      <c r="A33" s="20" t="inlineStr">
+    <row r="33" ht="72" customHeight="1" s="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>Main_UI_032</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>移动-路径寻路（有障碍物但有岔路）</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E33" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F33" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G33" s="20" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H33" s="20" t="inlineStr">
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>1.点击左鼠标去可以去的地形但前方有障碍物，但是有分路口可以到达
 2.观察角色是否移动到该地点</t>
         </is>
       </c>
-      <c r="I33" s="20" t="inlineStr">
+      <c r="I33" s="11" t="inlineStr">
         <is>
           <t>角色自动寻找可以前往的路线抵达该地点</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="42" customHeight="1" s="1">
-      <c r="A34" s="20" t="inlineStr">
+    <row r="34" ht="72" customHeight="1" s="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>Main_UI_033</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C34" s="20" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>移动-死胡同阻挡</t>
         </is>
       </c>
-      <c r="D34" s="22" t="inlineStr">
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E34" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F34" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G34" s="20" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H34" s="20" t="inlineStr">
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>1.点击左鼠标去不可以去的地形但地形两边均有障碍物
 2.观察角色是否移动到该地点</t>
         </is>
       </c>
-      <c r="I34" s="20" t="inlineStr">
+      <c r="I34" s="11" t="inlineStr">
         <is>
           <t>角色走到离死胡同最近的地方停下，并未进入到死胡同</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1" s="1">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="35" ht="72" customHeight="1" s="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>Main_UI_034</t>
         </is>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>移动-切换为WASD键盘模式</t>
         </is>
       </c>
-      <c r="D35" s="22" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E35" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F35" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G35" s="20" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H35" s="20" t="inlineStr">
+      <c r="H35" s="11" t="inlineStr">
         <is>
           <t>1.更改移动方式
 2.进入游戏内是否更改了移动方式</t>
         </is>
       </c>
-      <c r="I35" s="20" t="inlineStr">
+      <c r="I35" s="11" t="inlineStr">
         <is>
           <t>角色移动方式更改，现在由键盘WASD键控制人物的移动</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1" s="1">
-      <c r="A36" s="20" t="inlineStr">
+    <row r="36" ht="72" customHeight="1" s="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Main_UI_035</t>
         </is>
       </c>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C36" s="20" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>移动-WASD四方向控制</t>
         </is>
       </c>
-      <c r="D36" s="22" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E36" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F36" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G36" s="20" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H36" s="20" t="inlineStr">
+      <c r="H36" s="11" t="inlineStr">
         <is>
           <t>1.依次点击WASD
 2.观察角色是否正确方向移动</t>
         </is>
       </c>
-      <c r="I36" s="20" t="inlineStr">
+      <c r="I36" s="11" t="inlineStr">
         <is>
           <t>W对应人物的向上运动，A对应人物的向左运动，S对应人物的向下运动，D对应人物的向右运动，</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1" s="1">
-      <c r="A37" s="20" t="inlineStr">
+    <row r="37" ht="72" customHeight="1" s="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>Main_UI_036</t>
         </is>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>角色移动</t>
         </is>
       </c>
-      <c r="C37" s="20" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>移动-键盘模式遇障碍物阻挡</t>
         </is>
       </c>
-      <c r="D37" s="22" t="inlineStr">
+      <c r="D37" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E37" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F37" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G37" s="20" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H37" s="20" t="inlineStr">
+      <c r="H37" s="11" t="inlineStr">
         <is>
           <t>1.当人物遇见不可通过地形时
 2.持续按WASD观察角色是否移动到非地形区域</t>
         </is>
       </c>
-      <c r="I37" s="20" t="inlineStr">
+      <c r="I37" s="11" t="inlineStr">
         <is>
           <t>角色在非移动区域停止不同，可以后退离开，但不可以继续前进</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1" s="1">
-      <c r="A38" s="20" t="inlineStr">
+    <row r="38" ht="72" customHeight="1" s="1">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>Main_UI_037</t>
         </is>
       </c>
-      <c r="B38" s="20" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>新手引导</t>
         </is>
       </c>
-      <c r="C38" s="20" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>新手引导</t>
         </is>
       </c>
-      <c r="D38" s="22" t="inlineStr">
+      <c r="D38" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E38" s="20" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>体验测试</t>
         </is>
       </c>
-      <c r="F38" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G38" s="20" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
         <is>
           <t>进入游戏内</t>
         </is>
       </c>
-      <c r="H38" s="20" t="inlineStr">
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>1.观看新手引导
 2.按照新手引导做出相应的动作</t>
         </is>
       </c>
-      <c r="I38" s="20" t="inlineStr">
+      <c r="I38" s="11" t="inlineStr">
         <is>
           <t>1. 新手引导内容完整、步骤清晰
 2. 引导箭头或高亮提示正确指向交互目标
@@ -3017,493 +2988,1939 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="28" customHeight="1" s="1">
-      <c r="A39" s="20" t="inlineStr">
+    <row r="39" ht="72" customHeight="1" s="1">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Main_UI_038</t>
         </is>
       </c>
-      <c r="B39" s="20" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C39" s="20" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>基础攻击</t>
         </is>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E39" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F39" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G39" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H39" s="20" t="inlineStr">
-        <is>
-          <t>1.点击鼠标右键（血刃）（在键盘移动下）
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>1.点击鼠标右键（在键盘移动下）
 2.观察是否做出攻击动作并消耗MP</t>
         </is>
       </c>
-      <c r="I39" s="20" t="inlineStr">
+      <c r="I39" s="11" t="inlineStr">
         <is>
           <t>1.成功做出攻击动作
 2.并消耗相应的MP</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="42" customHeight="1" s="1">
-      <c r="A40" s="20" t="inlineStr">
+    <row r="40" ht="72" customHeight="1" s="1">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>Main_UI_039</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C40" s="20" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>基础攻击</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E40" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F40" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G40" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H40" s="20" t="inlineStr">
-        <is>
-          <t>1.持续点击鼠标右键（血刃）（在键盘移动下）
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>1.持续点击鼠标右键（在键盘移动下）
 2.观察是否做出攻击动作并消耗MP</t>
         </is>
       </c>
-      <c r="I40" s="20" t="inlineStr">
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>1.持续做出攻击动作
 2.并持续消耗相应的MP</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1" s="1">
-      <c r="A41" s="20" t="inlineStr">
+    <row r="41" ht="72" customHeight="1" s="1">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Main_UI_040</t>
         </is>
       </c>
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C41" s="20" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>基础攻击</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E41" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F41" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G41" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H41" s="20" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>选择职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
         <is>
           <t>1.点击鼠标右键（在键盘移动下）
 2.攻击尸观察伤害是否正常</t>
         </is>
       </c>
-      <c r="I41" s="20" t="inlineStr">
+      <c r="I41" s="11" t="inlineStr">
         <is>
           <t>1.攻击动画正常
 2.敌人受到伤害并显示伤害数字</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="42" customHeight="1" s="1">
-      <c r="A42" s="20" t="inlineStr">
+    <row r="42" ht="72" customHeight="1" s="1">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>Main_UI_041</t>
         </is>
       </c>
-      <c r="B42" s="20" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C42" s="20" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
         <is>
           <t>基础攻击</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D42" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E42" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F42" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G42" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H42" s="20" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
         <is>
           <t>1.击败血尸
 2.观察血尸是否播放击败动画
 3.观察经验和金币或者战利品是否增加</t>
         </is>
       </c>
-      <c r="I42" s="20" t="inlineStr">
+      <c r="I42" s="11" t="inlineStr">
         <is>
           <t>1.血尸播放击败动画
 2.血尸击败后掉落金币与经验值XP</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="28" customHeight="1" s="1">
-      <c r="A43" s="20" t="inlineStr">
+    <row r="43" ht="72" customHeight="1" s="1">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Main_UI_042</t>
         </is>
       </c>
-      <c r="B43" s="20" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C43" s="20" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>Shift+右键攻击（鼠标模式下）</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E43" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F43" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G43" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H43" s="20" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
         <is>
           <t>1.点击Shift+鼠标右键（在鼠标移动下）
 2.打血尸观察伤害是否正常</t>
         </is>
       </c>
-      <c r="I43" s="20" t="inlineStr">
+      <c r="I43" s="11" t="inlineStr">
         <is>
           <t>1. 攻击动画正常
 2. 敌人受到伤害并显示伤害数字</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="28" customHeight="1" s="1">
-      <c r="A44" s="20" t="inlineStr">
+    <row r="44" ht="72" customHeight="1" s="1">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>Main_UI_043</t>
         </is>
       </c>
-      <c r="B44" s="20" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C44" s="20" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
         <is>
           <t>左键攻击（鼠标模式下）</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E44" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F44" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G44" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H44" s="20" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
         <is>
           <t>1.点击鼠标左键（在鼠标移动下）
 2.打血尸观察伤害是否正常</t>
         </is>
       </c>
-      <c r="I44" s="20" t="inlineStr">
+      <c r="I44" s="11" t="inlineStr">
         <is>
           <t>1. 攻击动画正常
 2. 敌人受到伤害并显示伤害数字</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="14.5" customHeight="1" s="1">
-      <c r="A45" s="20" t="inlineStr">
+    <row r="45" ht="72" customHeight="1" s="1">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>Main_UI_044</t>
         </is>
       </c>
-      <c r="B45" s="20" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C45" s="20" t="inlineStr">
+      <c r="C45" s="11" t="inlineStr">
         <is>
           <t>技能图标拖拽到角色身上</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>异常测试</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G45" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H45" s="20" t="inlineStr">
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>选择职业职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>长按技能拖动到角色身上</t>
         </is>
       </c>
-      <c r="I45" s="20" t="inlineStr">
+      <c r="I45" s="11" t="inlineStr">
         <is>
           <t>技能图标应返回原位或取消拖拽状态，角色不应执行任何攻击动作。若技能消失且角色不攻击则属于界面交互Bug</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="28" customHeight="1" s="1">
-      <c r="A46" s="20" t="inlineStr">
+    <row r="46" ht="72" customHeight="1" s="1">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>Main_UI_045</t>
         </is>
       </c>
-      <c r="B46" s="20" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C46" s="20" t="inlineStr">
+      <c r="C46" s="11" t="inlineStr">
         <is>
           <t>受到攻击</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D46" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E46" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F46" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G46" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H46" s="20" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>1.受到血尸攻击
 2.观察是否HP是否减少</t>
         </is>
       </c>
-      <c r="I46" s="20" t="inlineStr">
+      <c r="I46" s="11" t="inlineStr">
         <is>
           <t>1.血尸攻击动画正常
 2.角色HP减少</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="14.5" customHeight="1" s="1">
-      <c r="A47" s="20" t="inlineStr">
+    <row r="47" ht="72" customHeight="1" s="1">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>Main_UI_046</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C47" s="20" t="inlineStr">
+      <c r="C47" s="11" t="inlineStr">
         <is>
           <t>HP自动回复机制</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E47" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F47" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G47" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H47" s="20" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
         <is>
           <t>当角色HP值不是满的情况下观察HP是否回复</t>
         </is>
       </c>
-      <c r="I47" s="20" t="inlineStr">
+      <c r="I47" s="11" t="inlineStr">
         <is>
           <t>角色HP速率与介绍一致正常回复，回复到上限不回复</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="14.5" customHeight="1" s="1">
-      <c r="A48" s="20" t="inlineStr">
+    <row r="48" ht="72" customHeight="1" s="1">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>Main_UI_047</t>
         </is>
       </c>
-      <c r="B48" s="20" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>战斗系统</t>
         </is>
       </c>
-      <c r="C48" s="20" t="inlineStr">
+      <c r="C48" s="11" t="inlineStr">
         <is>
           <t>MP自动回复机制</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E48" s="20" t="inlineStr">
-        <is>
-          <t>功能测试</t>
-        </is>
-      </c>
-      <c r="F48" s="20" t="inlineStr">
-        <is>
-          <t>Flare 1.15</t>
-        </is>
-      </c>
-      <c r="G48" s="20" t="inlineStr">
-        <is>
-          <t>进入游戏内</t>
-        </is>
-      </c>
-      <c r="H48" s="20" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
         <is>
           <t>当角色MP值不是满的情况下观察MP是否回复</t>
         </is>
       </c>
-      <c r="I48" s="20" t="inlineStr">
+      <c r="I48" s="11" t="inlineStr">
         <is>
           <t>角色MP速率与介绍一致正常回复，回复到上限不回复</t>
         </is>
       </c>
     </row>
+    <row r="49" ht="72" customHeight="1" s="1">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_048</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>装备掉落</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>1.角色正常击败敌人
+2.观察装备是否掉落和是否可以拾取</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>敌人掉落装备并可以正常拾取到背包</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="72" customHeight="1" s="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_049</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>装备穿戴</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入背包界面
+2. 穿戴或者脱下装备
+3. 观察角色的属性变化与外观变化</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>1. 穿戴装备后角色属性正确提升，外观改变
+2. 卸下装备后属性回归到初始状态，外观恢复</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="72" customHeight="1" s="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_050</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>装备属性</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>1.进入背包界面
+2.鼠标悬停在不同品质的装备上
+3.观察是否有装备的基本名称，售价，等级，加成属性</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>不同品质的装备表现不同：边框颜色、名称颜色、售价、基础属性、等级要求均有差异</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="72" customHeight="1" s="1">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_051</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>装备穿戴</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入背包界面
+2. 长按装备拖出装备区（模拟用户异常操作）
+3. 观察装备是否显示在地图上</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>正常情况下装备应返回原位或提示不可拖出，装备不应丢失。若装备掉落在地图上可重新拾取</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="72" customHeight="1" s="1">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_052</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>后台切换</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>1进入背包界面
+2.正确穿戴装备
+3.切换后台再切回
+4.观察属性是否发生改变</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr">
+        <is>
+          <t>切换后台发现属性正常无异常状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1" s="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_053</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>装备职业限制</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>创建不同两个存档【力士】【法师】</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>1.将【力士】装备切换至【法师】装备
+2.观察是否可以正常穿戴</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
+          <t>有职业限制的装备不可穿戴，显示职业要求，没有职业要求的各职业都可以穿戴</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1" s="1">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_054</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>装备对比</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>进入背包界面</t>
+        </is>
+      </c>
+      <c r="H55" s="11" t="inlineStr">
+        <is>
+          <t>鼠标悬停在装备上，观察是否与
+身上所穿戴的装备进行对比</t>
+        </is>
+      </c>
+      <c r="I55" s="11" t="inlineStr">
+        <is>
+          <t>装备进行对比，不同品质的装备显示边框不同</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="72" customHeight="1" s="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_055</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>装备切换</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>进入背包界面</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="inlineStr">
+        <is>
+          <t>1.准备2件有属性差异的装备（一件已经装备）
+2.切换穿戴
+3.观察角色属性是否发生改变</t>
+        </is>
+      </c>
+      <c r="I56" s="11" t="inlineStr">
+        <is>
+          <t>不同装备穿戴，旧属性旧外观移除属性，新属性与外观添加</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="72" customHeight="1" s="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_056</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>卸下装备</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>进入背包界面</t>
+        </is>
+      </c>
+      <c r="H57" s="11" t="inlineStr">
+        <is>
+          <t>所有装备移除，裸装备观察属性</t>
+        </is>
+      </c>
+      <c r="I57" s="11" t="inlineStr">
+        <is>
+          <t>装备属性移除，回到初始属性</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="72" customHeight="1" s="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_057</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>背包交互</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>1.点击I键或者鼠标点击背包图标
+2.观察是否进行交互</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
+        <is>
+          <t>I键与点击背包均可以打开背包界面</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="72" customHeight="1" s="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_058</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>物品拾取</t>
+        </is>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>选择任意职业进入游戏内</t>
+        </is>
+      </c>
+      <c r="H59" s="11" t="inlineStr">
+        <is>
+          <t>击败血尸，观察地上是否有掉落物，走过去拾取，观察背包是否增加该物品</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>背包增加掉落物</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="72" customHeight="1" s="1">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_059</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>使用消耗品</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>HP/MP不满时</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>打开背包使用充能药水和治疗药水，观察药水是否减少，MP/HP是否回复</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>背包内药水减少,MP/HP回复正常</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="72" customHeight="1" s="1">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_060</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>UI界面</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>打开背包</t>
+        </is>
+      </c>
+      <c r="H61" s="11" t="inlineStr">
+        <is>
+          <t>观察检查背包格子数量、行列间距是否与设计合理。在深色/浅色模式下，物品图标、数量角标、品质边框是否显示清晰。</t>
+        </is>
+      </c>
+      <c r="I61" s="11" t="inlineStr">
+        <is>
+          <t>背包UI界面一切正常</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="72" customHeight="1" s="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_061</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>UX界面</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>打开背包</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>通过不同排序（Text/Quality），观察物品是否正常排序</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>物品按照所选择的排序方式进行排序</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="72" customHeight="1" s="1">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_062</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="inlineStr">
+        <is>
+          <t>物品丢弃</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G63" s="11" t="inlineStr">
+        <is>
+          <t>打开背包</t>
+        </is>
+      </c>
+      <c r="H63" s="11" t="inlineStr">
+        <is>
+          <t>拖拽物品丢弃，观察背包内是否消失</t>
+        </is>
+      </c>
+      <c r="I63" s="11" t="inlineStr">
+        <is>
+          <t>背包物品消失</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="72" customHeight="1" s="1">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_063</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>物品堆叠-同类物品</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>背包中有至少1瓶药水</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>1. 继续拾取同种药水
+2. 观察背包显示</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>同类物品自动堆叠，显示数量叠加（如 x2 变 x3），占用同一格子</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="72" customHeight="1" s="1">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_064</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="inlineStr">
+        <is>
+          <t>物品堆叠-达到上限</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>边界测试</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G65" s="11" t="inlineStr">
+        <is>
+          <t>背包中某物品堆叠已满</t>
+        </is>
+      </c>
+      <c r="H65" s="11" t="inlineStr">
+        <is>
+          <t>1. 继续拾取同种物品
+2. 观察背包变化</t>
+        </is>
+      </c>
+      <c r="I65" s="11" t="inlineStr">
+        <is>
+          <t>新拾取物品另起一格，原有堆叠不变，无物品丢失</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="72" customHeight="1" s="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_065</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C66" s="11" t="inlineStr">
+        <is>
+          <t>背包满时拾取</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>边界测试</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr">
+        <is>
+          <t>背包所有格子已满</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>1. 击败怪物
+2. 观察掉落物能否拾取</t>
+        </is>
+      </c>
+      <c r="I66" s="11" t="inlineStr">
+        <is>
+          <t>弹出背包已满提示，物品无法拾取或掉落在原地可稍后拾取</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="72" customHeight="1" s="1">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_066</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C67" s="11" t="inlineStr">
+        <is>
+          <t>右键快捷穿戴装备</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G67" s="11" t="inlineStr">
+        <is>
+          <t>背包中有未穿戴的装备</t>
+        </is>
+      </c>
+      <c r="H67" s="11" t="inlineStr">
+        <is>
+          <t>1. 右键点击背包中的装备
+2. 观察是否自动穿戴到对应槽位</t>
+        </is>
+      </c>
+      <c r="I67" s="11" t="inlineStr">
+        <is>
+          <t>装备自动穿戴到对应槽位，属性正确更新</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="72" customHeight="1" s="1">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_067</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>背包系统</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>物品丢弃-确认机制</t>
+        </is>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>异常测试</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G68" s="11" t="inlineStr">
+        <is>
+          <t>打开背包</t>
+        </is>
+      </c>
+      <c r="H68" s="11" t="inlineStr">
+        <is>
+          <t>1. 拖拽物品丢弃
+2. 观察是否有确认弹窗</t>
+        </is>
+      </c>
+      <c r="I68" s="11" t="inlineStr">
+        <is>
+          <t>有确认弹窗（如“确定丢弃？”），确认后物品消失，取消则物品保留</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="72" customHeight="1" s="1">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_068</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>空装备栏状态</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G69" s="11" t="inlineStr">
+        <is>
+          <t>创建新角色，未穿戴任何装备</t>
+        </is>
+      </c>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>1. 打开角色面板
+2. 观察各装备槽位显示</t>
+        </is>
+      </c>
+      <c r="I69" s="11" t="inlineStr">
+        <is>
+          <t>各槽位显示为空，对应属性为角色基础值，无异常显示</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="72" customHeight="1" s="1">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_069</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>装备系统</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>多件同部位装备切换</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G70" s="11" t="inlineStr">
+        <is>
+          <t>背包中有2件以上同部位装备</t>
+        </is>
+      </c>
+      <c r="H70" s="11" t="inlineStr">
+        <is>
+          <t>1. 右键穿戴装备A
+2. 右键穿戴装备B
+3. 观察面板变化</t>
+        </is>
+      </c>
+      <c r="I70" s="11" t="inlineStr">
+        <is>
+          <t>装备B替换装备A，A的属性被移除，B的属性正确叠加</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="72" customHeight="1" s="1">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_070</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>设置系统</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="inlineStr">
+        <is>
+          <t>音量设置-生效</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="inlineStr">
+        <is>
+          <t>游戏已启动</t>
+        </is>
+      </c>
+      <c r="H71" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入设置
+2. 调整音量滑块到不同值
+3. 观察实际音量变化</t>
+        </is>
+      </c>
+      <c r="I71" s="11" t="inlineStr">
+        <is>
+          <t>音量随滑块调整正确变化，静音时完全无声</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="72" customHeight="1" s="1">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_071</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>设置系统</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>画面设置-全屏/窗口切换</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G72" s="11" t="inlineStr">
+        <is>
+          <t>游戏已启动</t>
+        </is>
+      </c>
+      <c r="H72" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入设置
+2. 切换全屏/窗口模式
+3. 观察画面变化</t>
+        </is>
+      </c>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>模式切换成功，游戏画面正常渲染，无黑边或拉伸</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="72" customHeight="1" s="1">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_072</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>设置系统</t>
+        </is>
+      </c>
+      <c r="C73" s="11" t="inlineStr">
+        <is>
+          <t>按键设置-自定义键位</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>游戏已启动</t>
+        </is>
+      </c>
+      <c r="H73" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入设置
+2. 修改按键绑定（如移动键WASD改为IJKL）
+3. 保存并应用</t>
+        </is>
+      </c>
+      <c r="I73" s="11" t="inlineStr">
+        <is>
+          <t>新键位生效，旧键位失效，无冲突提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="72" customHeight="1" s="1">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_073</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>死亡系统</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>未勾选不可复活-死亡</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>创建角色时未勾选死亡不可复活</t>
+        </is>
+      </c>
+      <c r="H74" s="11" t="inlineStr">
+        <is>
+          <t>1. 进入游戏让角色死亡
+2. 观察死亡界面选项</t>
+        </is>
+      </c>
+      <c r="I74" s="11" t="inlineStr">
+        <is>
+          <t>死亡后显示复活选项，点击复活后角色在安全点重生，属性正常</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="72" customHeight="1" s="1">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_074</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>死亡系统</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
+          <t>死亡-装备/物品保留</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>角色已有装备和背包物品</t>
+        </is>
+      </c>
+      <c r="H75" s="11" t="inlineStr">
+        <is>
+          <t>1. 让角色死亡
+2. 复活后检查装备和背包</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>装备和背包物品与死亡前一致，无丢失</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="72" customHeight="1" s="1">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_075</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>升级系统</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>击杀获得经验</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>创建新角色进入游戏</t>
+        </is>
+      </c>
+      <c r="H76" s="11" t="inlineStr">
+        <is>
+          <t>1. 击杀怪物
+2. 观察经验值变化</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>击杀怪物后经验值增加，有经验获取反馈提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="72" customHeight="1" s="1">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_076</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>升级系统</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>升级-属性/技能变化</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>角色经验满即将升级</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="inlineStr">
+        <is>
+          <t>1. 击杀怪物触发升级
+2. 观察升级前后对比</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>基础属性提升，可能获得技能点，升级动画或提示正常显示</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="72" customHeight="1" s="1">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>Main_UI_077</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>升级系统</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>升级-属性分配</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>功能测试</t>
+        </is>
+      </c>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>Flare 1.15</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>角色升级后获得属性点</t>
+        </is>
+      </c>
+      <c r="H78" s="11" t="inlineStr">
+        <is>
+          <t>1. 打开角色面板
+2. 分配属性点
+3. 观察属性变化</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>属性点可用且分配后对应属性正确提升，保存后再次登录属性保留</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:I78"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>